<commit_message>
various changes and updates
</commit_message>
<xml_diff>
--- a/VaydeerMacropadTemplate.xlsx
+++ b/VaydeerMacropadTemplate.xlsx
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$G$10</definedName>
+  </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>C+5</t>
   </si>
@@ -49,89 +52,59 @@
     <t>C+B</t>
   </si>
   <si>
-    <t>S+F5</t>
-  </si>
-  <si>
-    <t>F5</t>
-  </si>
-  <si>
     <t>JS Run</t>
   </si>
   <si>
     <t>F8</t>
   </si>
   <si>
-    <t>F10</t>
-  </si>
-  <si>
-    <t>Run Dbg</t>
-  </si>
-  <si>
-    <t>Stop Dbg</t>
-  </si>
-  <si>
-    <t>Debug Test</t>
-  </si>
-  <si>
-    <t>Run Teset</t>
-  </si>
-  <si>
     <t>Dbg Over</t>
   </si>
   <si>
     <t>Dbg Into</t>
   </si>
   <si>
-    <t>F11</t>
-  </si>
-  <si>
-    <t>Mic Toggle</t>
-  </si>
-  <si>
-    <t>Share Scrn</t>
-  </si>
-  <si>
-    <t>C+E</t>
-  </si>
-  <si>
-    <t>End Mtg</t>
-  </si>
-  <si>
-    <t>C+H</t>
-  </si>
-  <si>
-    <t>VS</t>
-  </si>
-  <si>
-    <t>Win+3</t>
-  </si>
-  <si>
-    <t>SqlEd</t>
-  </si>
-  <si>
-    <t>Win+4</t>
-  </si>
-  <si>
-    <t>C+S+K</t>
-  </si>
-  <si>
-    <t>TeamsClap</t>
-  </si>
-  <si>
-    <t>TypeAdmin</t>
-  </si>
-  <si>
-    <t>AdminPwd</t>
-  </si>
-  <si>
-    <t>CorpPwd</t>
+    <t>Close Win</t>
+  </si>
+  <si>
+    <t>Type Admin</t>
+  </si>
+  <si>
+    <t>Run Test</t>
+  </si>
+  <si>
+    <t>Dbg Test</t>
+  </si>
+  <si>
+    <t>Type Admin Pwd</t>
+  </si>
+  <si>
+    <t>Type Dev Supp Pwd</t>
+  </si>
+  <si>
+    <t>Type My Pwd</t>
+  </si>
+  <si>
+    <t>S+F9</t>
+  </si>
+  <si>
+    <t>DbgQckWtch</t>
+  </si>
+  <si>
+    <t>VS VM</t>
+  </si>
+  <si>
+    <t>F12</t>
+  </si>
+  <si>
+    <t>ExitApp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,6 +121,25 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -173,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -362,11 +354,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -443,6 +474,54 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,7 +726,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>4601</xdr:colOff>
+      <xdr:colOff>4602</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>457200</xdr:rowOff>
     </xdr:to>
@@ -997,10 +1076,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="47.28515625" customWidth="1"/>
+    <col min="4" max="4" width="42.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1032,34 +1111,38 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
       <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>29</v>
+        <v>4</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
+      <c r="A4" s="5" t="s">
+        <v>3</v>
+      </c>
       <c r="B4" s="6" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="E4" s="37"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="29"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
@@ -1082,44 +1165,28 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>23</v>
-      </c>
+      <c r="E6" s="39"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="28"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>4</v>
-      </c>
+      <c r="A7" s="11"/>
       <c r="B7" s="12" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>24</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E7" s="40"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="29"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1143,45 +1210,48 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>16</v>
+      <c r="F9" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="24" t="s">
-        <v>20</v>
-      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="24"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="32"/>
     </row>
+    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+  </mergeCells>
   <pageMargins left="0.25" right="0" top="0.25" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>